<commit_message>
Aggiungi indirizzi ai dizionari
</commit_message>
<xml_diff>
--- a/GUI.WinForms/Resources/StemDictionaries.xlsx
+++ b/GUI.WinForms/Resources/StemDictionaries.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucav\source\repos\bitbucket\StemDeviceManager\GUI.Windows\Resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucav\source\repos\bitbucket\Stem.ButtonPanel.Tester\GUI.WinForms\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08B259F7-01CF-4E8A-8947-2470824AFB2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68597906-5484-47A0-A582-BC5105491074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3980" uniqueCount="1037">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3983" uniqueCount="1040">
   <si>
     <t>NOME COMANDO</t>
   </si>
@@ -4212,6 +4212,15 @@
   </si>
   <si>
     <t>0x000C0103</t>
+  </si>
+  <si>
+    <t>0x1FFFFFFF</t>
+  </si>
+  <si>
+    <t>0x00000001</t>
+  </si>
+  <si>
+    <t>0xFFFFFFFF</t>
   </si>
 </sst>
 </file>
@@ -54730,31 +54739,27 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC9196D1-9EE6-4F09-A35C-2208B4458743}">
-  <dimension ref="A1:T35"/>
+  <dimension ref="A1:V35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" customWidth="1"/>
-    <col min="3" max="3" width="23.42578125" customWidth="1"/>
+    <col min="2" max="3" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.5703125" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.28515625" customWidth="1"/>
-    <col min="10" max="10" width="14.28515625" customWidth="1"/>
+    <col min="9" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="41" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="17" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.140625" customWidth="1"/>
-    <col min="17" max="17" width="16" customWidth="1"/>
-    <col min="18" max="18" width="16.5703125" customWidth="1"/>
-    <col min="19" max="19" width="15.42578125" customWidth="1"/>
+    <col min="16" max="17" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="22" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="104" t="s">
         <v>765</v>
       </c>
@@ -54769,7 +54774,7 @@
       <c r="J1" s="104"/>
       <c r="K1" s="3"/>
     </row>
-    <row r="2" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>773</v>
       </c>
@@ -54827,8 +54832,17 @@
       <c r="S2" s="1" t="s">
         <v>1033</v>
       </c>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="T2" s="1" t="s">
+        <v>1037</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>1038</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>1039</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>603</v>
       </c>
@@ -54873,7 +54887,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="39" t="s">
         <v>88</v>
       </c>
@@ -54897,7 +54911,7 @@
       <c r="S4" s="102"/>
       <c r="T4" s="103"/>
     </row>
-    <row r="5" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="37" t="str">
         <f>IF('DATI LOGICI'!A3&lt;&gt;"",'DATI LOGICI'!A3,"")</f>
         <v>Firmware macchina</v>
@@ -54937,7 +54951,7 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="37" t="str">
         <f>IF('DATI LOGICI'!A4&lt;&gt;"",'DATI LOGICI'!A4,"")</f>
         <v>Firmware scheda</v>
@@ -54986,7 +55000,7 @@
       <c r="S6" s="102"/>
       <c r="T6" s="103"/>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="54" t="str">
         <f>IF('DATI LOGICI'!A5&lt;&gt;"",'DATI LOGICI'!A5,"")</f>
         <v>Modello</v>
@@ -55025,7 +55039,7 @@
       </c>
       <c r="J7" s="3"/>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" s="54" t="str">
         <f>IF('DATI LOGICI'!A6&lt;&gt;"",'DATI LOGICI'!A6,"")</f>
         <v>Matricola</v>
@@ -55064,7 +55078,7 @@
       </c>
       <c r="J8" s="3"/>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" s="54" t="str">
         <f>IF('DATI LOGICI'!A7&lt;&gt;"",'DATI LOGICI'!A7,"")</f>
         <v>Tipo scheda</v>
@@ -55102,7 +55116,7 @@
       </c>
       <c r="J9" s="3"/>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" s="54" t="str">
         <f>IF('DATI LOGICI'!A8&lt;&gt;"",'DATI LOGICI'!A8,"")</f>
         <v>Stato</v>
@@ -55141,7 +55155,7 @@
       </c>
       <c r="J10" s="3"/>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" s="54" t="str">
         <f>IF('DATI LOGICI'!A9&lt;&gt;"",'DATI LOGICI'!A9,"")</f>
         <v>Allarmi</v>
@@ -55182,7 +55196,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" s="54" t="str">
         <f>IF('DATI LOGICI'!A10&lt;&gt;"",'DATI LOGICI'!A10,"")</f>
         <v>Comandi</v>
@@ -55221,7 +55235,7 @@
       </c>
       <c r="J12" s="1"/>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" s="54" t="str">
         <f>IF('DATI LOGICI'!A11&lt;&gt;"",'DATI LOGICI'!A11,"")</f>
         <v>Temperatura scheda</v>
@@ -55260,7 +55274,7 @@
       </c>
       <c r="J13" s="1"/>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" s="54" t="str">
         <f>IF('DATI LOGICI'!A12&lt;&gt;"",'DATI LOGICI'!A12,"")</f>
         <v>Secondi lavoro motore parziale</v>
@@ -55299,7 +55313,7 @@
       </c>
       <c r="J14" s="1"/>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" s="54" t="str">
         <f>IF('DATI LOGICI'!A13&lt;&gt;"",'DATI LOGICI'!A13,"")</f>
         <v>Secondi lavoro motore totale</v>
@@ -55338,7 +55352,7 @@
       </c>
       <c r="J15" s="1"/>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" s="54" t="str">
         <f>IF('DATI LOGICI'!A14&lt;&gt;"",'DATI LOGICI'!A14,"")</f>
         <v>Cicli complessivi parziale</v>

</xml_diff>